<commit_message>
output file names corrections, updated xls
</commit_message>
<xml_diff>
--- a/QuickRegressionTesting5.xlsx
+++ b/QuickRegressionTesting5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://thermofisher-my.sharepoint.com/personal/aswathy_n_thermofisher_com/Documents/Aswathy (1)/My_learning/programming_learning/GL_AIML/KeyAreas/GitHub_CICDLearning/RegressionScripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{27A84F89-77DE-E94A-B7B2-4ADE76FB0224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{287D984B-1D2B-8344-9837-7C3E531BB795}"/>
+  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{27A84F89-77DE-E94A-B7B2-4ADE76FB0224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{998848BB-5BD6-874C-B37D-66E1C515465F}"/>
   <bookViews>
-    <workbookView xWindow="44860" yWindow="2860" windowWidth="27720" windowHeight="16940" firstSheet="3" activeTab="4" xr2:uid="{F1B42ADB-BE16-DF45-8356-FD35A5FE073C}"/>
+    <workbookView xWindow="44860" yWindow="2860" windowWidth="27720" windowHeight="16940" firstSheet="3" activeTab="3" xr2:uid="{F1B42ADB-BE16-DF45-8356-FD35A5FE073C}"/>
   </bookViews>
   <sheets>
     <sheet name="URLSheet" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="349">
   <si>
     <t>URL</t>
   </si>
@@ -3526,7 +3526,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3615,28 +3615,44 @@
     <xf numFmtId="49" fontId="15" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3661,37 +3677,22 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6367,13 +6368,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59DE326C-3520-BF47-B048-078953A62B20}">
-  <dimension ref="A1:C287"/>
+  <dimension ref="A1:E287"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="47.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -6384,1599 +6385,1651 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="128" customHeight="1">
-      <c r="A2" s="36" t="s">
+    <row r="2" spans="1:5" ht="128" customHeight="1">
+      <c r="A2" s="46" t="s">
         <v>185</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="49" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="96" customHeight="1">
-      <c r="A3" s="37"/>
-      <c r="B3" s="35"/>
-      <c r="C3" s="59"/>
-    </row>
-    <row r="4" spans="1:3" ht="160" customHeight="1">
-      <c r="A4" s="36" t="s">
+    <row r="3" spans="1:5" ht="96" customHeight="1">
+      <c r="A3" s="48"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="50"/>
+    </row>
+    <row r="4" spans="1:5" ht="160" customHeight="1">
+      <c r="A4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C4" s="60" t="s">
+      <c r="C4" s="51" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="37"/>
-      <c r="B5" s="35"/>
-      <c r="C5" s="61"/>
-    </row>
-    <row r="6" spans="1:3" ht="224" customHeight="1">
-      <c r="A6" s="36" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" s="48"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="52"/>
+    </row>
+    <row r="6" spans="1:5" ht="224" customHeight="1">
+      <c r="A6" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="60" t="s">
+      <c r="C6" s="51" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="37"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="61"/>
-    </row>
-    <row r="8" spans="1:3" ht="64" customHeight="1">
-      <c r="A8" s="36" t="s">
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="43" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="48"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="52"/>
+      <c r="E7" s="44"/>
+    </row>
+    <row r="8" spans="1:5" ht="64" customHeight="1">
+      <c r="A8" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="38"/>
-      <c r="C8" s="62" t="s">
+      <c r="B8" s="34"/>
+      <c r="C8" s="40" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="335" customHeight="1">
-      <c r="A9" s="39"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="63"/>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" s="39"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="63"/>
-    </row>
-    <row r="11" spans="1:3" ht="320" customHeight="1">
-      <c r="A11" s="39"/>
-      <c r="B11" s="34" t="s">
+    <row r="9" spans="1:5" ht="335" customHeight="1">
+      <c r="A9" s="47"/>
+      <c r="B9" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C11" s="63"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="64"/>
-    </row>
-    <row r="13" spans="1:3" ht="272" customHeight="1">
-      <c r="A13" s="36" t="s">
+      <c r="C9" s="41"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="47"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="41"/>
+    </row>
+    <row r="11" spans="1:5" ht="320" customHeight="1">
+      <c r="A11" s="47"/>
+      <c r="B11" s="44"/>
+      <c r="C11" s="41"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="48"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="42"/>
+    </row>
+    <row r="13" spans="1:5" ht="272" customHeight="1">
+      <c r="A13" s="46" t="s">
         <v>187</v>
       </c>
-      <c r="B13" s="38"/>
-      <c r="C13" s="62" t="s">
+      <c r="B13" s="44"/>
+      <c r="C13" s="40" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" s="39"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="63"/>
-    </row>
-    <row r="15" spans="1:3" ht="112" customHeight="1">
-      <c r="A15" s="39"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="63"/>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" s="39"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="63"/>
+    <row r="14" spans="1:5">
+      <c r="A14" s="47"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="41"/>
+    </row>
+    <row r="15" spans="1:5" ht="112" customHeight="1">
+      <c r="A15" s="47"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="41"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="47"/>
+      <c r="B16" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="41"/>
     </row>
     <row r="17" spans="1:3" ht="48" customHeight="1">
-      <c r="A17" s="39"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="63"/>
+      <c r="A17" s="47"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="41"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="39"/>
-      <c r="B18" s="34" t="s">
+      <c r="A18" s="47"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="41"/>
+    </row>
+    <row r="19" spans="1:3" ht="32" customHeight="1">
+      <c r="A19" s="48"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="42"/>
+    </row>
+    <row r="20" spans="1:3" ht="409.5" customHeight="1">
+      <c r="A20" s="46" t="s">
+        <v>188</v>
+      </c>
+      <c r="B20" s="44"/>
+      <c r="C20" s="40" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="47"/>
+      <c r="B21" s="44"/>
+      <c r="C21" s="41"/>
+    </row>
+    <row r="22" spans="1:3" ht="32" customHeight="1">
+      <c r="A22" s="47"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="41"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="47"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="41"/>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="47"/>
+      <c r="B24" s="44"/>
+      <c r="C24" s="41"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="47"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="41"/>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="47"/>
+      <c r="B26" s="44"/>
+      <c r="C26" s="41"/>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="47"/>
+      <c r="B27" s="44"/>
+      <c r="C27" s="41"/>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="47"/>
+      <c r="B28" s="44"/>
+      <c r="C28" s="41"/>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="47"/>
+      <c r="B29" s="44"/>
+      <c r="C29" s="41"/>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="47"/>
+      <c r="B30" s="45"/>
+      <c r="C30" s="41"/>
+    </row>
+    <row r="31" spans="1:3" ht="80" customHeight="1">
+      <c r="A31" s="47"/>
+      <c r="B31" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="63"/>
-    </row>
-    <row r="19" spans="1:3" ht="32" customHeight="1">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="64"/>
-    </row>
-    <row r="20" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A20" s="36" t="s">
-        <v>188</v>
-      </c>
-      <c r="B20" s="38"/>
-      <c r="C20" s="62" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="39"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="63"/>
-    </row>
-    <row r="22" spans="1:3" ht="32" customHeight="1">
-      <c r="A22" s="39"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="63"/>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="39"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="63"/>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="39"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="63"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="39"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="63"/>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="39"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="63"/>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" s="39"/>
-      <c r="B27" s="38"/>
-      <c r="C27" s="63"/>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" s="39"/>
-      <c r="B28" s="38"/>
-      <c r="C28" s="63"/>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" s="39"/>
-      <c r="B29" s="38"/>
-      <c r="C29" s="63"/>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="39"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="63"/>
-    </row>
-    <row r="31" spans="1:3" ht="80" customHeight="1">
-      <c r="A31" s="39"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="63"/>
+      <c r="C31" s="41"/>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" s="39"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="63"/>
+      <c r="A32" s="47"/>
+      <c r="B32" s="44"/>
+      <c r="C32" s="41"/>
     </row>
     <row r="33" spans="1:3" ht="64" customHeight="1">
-      <c r="A33" s="39"/>
-      <c r="B33" s="34" t="s">
+      <c r="A33" s="47"/>
+      <c r="B33" s="44"/>
+      <c r="C33" s="41"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="48"/>
+      <c r="B34" s="44"/>
+      <c r="C34" s="42"/>
+    </row>
+    <row r="35" spans="1:3" ht="306" customHeight="1">
+      <c r="A35" s="46" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="44"/>
+      <c r="C35" s="40" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="47"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="41"/>
+    </row>
+    <row r="37" spans="1:3" ht="32" customHeight="1">
+      <c r="A37" s="47"/>
+      <c r="B37" s="44"/>
+      <c r="C37" s="41"/>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="47"/>
+      <c r="B38" s="44"/>
+      <c r="C38" s="41"/>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="47"/>
+      <c r="B39" s="44"/>
+      <c r="C39" s="41"/>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="47"/>
+      <c r="B40" s="44"/>
+      <c r="C40" s="41"/>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="47"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="41"/>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="47"/>
+      <c r="B42" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="63"/>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" s="37"/>
-      <c r="B34" s="38"/>
-      <c r="C34" s="64"/>
-    </row>
-    <row r="35" spans="1:3" ht="306" customHeight="1">
-      <c r="A35" s="36" t="s">
-        <v>189</v>
-      </c>
-      <c r="B35" s="38"/>
-      <c r="C35" s="62" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" s="39"/>
-      <c r="B36" s="38"/>
-      <c r="C36" s="63"/>
-    </row>
-    <row r="37" spans="1:3" ht="32" customHeight="1">
-      <c r="A37" s="39"/>
-      <c r="B37" s="38"/>
-      <c r="C37" s="63"/>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="39"/>
-      <c r="B38" s="38"/>
-      <c r="C38" s="63"/>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" s="39"/>
-      <c r="B39" s="38"/>
-      <c r="C39" s="63"/>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" s="39"/>
-      <c r="B40" s="38"/>
-      <c r="C40" s="63"/>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" s="39"/>
-      <c r="B41" s="38"/>
-      <c r="C41" s="63"/>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" s="39"/>
-      <c r="B42" s="38"/>
-      <c r="C42" s="63"/>
+      <c r="C42" s="41"/>
     </row>
     <row r="43" spans="1:3">
-      <c r="A43" s="39"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="63"/>
+      <c r="A43" s="47"/>
+      <c r="B43" s="44"/>
+      <c r="C43" s="41"/>
     </row>
     <row r="44" spans="1:3">
-      <c r="A44" s="39"/>
-      <c r="B44" s="34" t="s">
+      <c r="A44" s="47"/>
+      <c r="B44" s="44"/>
+      <c r="C44" s="41"/>
+    </row>
+    <row r="45" spans="1:3" ht="64" customHeight="1">
+      <c r="A45" s="48"/>
+      <c r="B45" s="44"/>
+      <c r="C45" s="42"/>
+    </row>
+    <row r="46" spans="1:3" ht="409.5" customHeight="1">
+      <c r="A46" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="B46" s="44"/>
+      <c r="C46" s="40" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="64" customHeight="1">
+      <c r="A47" s="47"/>
+      <c r="B47" s="44"/>
+      <c r="C47" s="41"/>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="47"/>
+      <c r="B48" s="44"/>
+      <c r="C48" s="41"/>
+    </row>
+    <row r="49" spans="1:3" ht="48" customHeight="1">
+      <c r="A49" s="47"/>
+      <c r="B49" s="44"/>
+      <c r="C49" s="41"/>
+    </row>
+    <row r="50" spans="1:3" ht="48" customHeight="1">
+      <c r="A50" s="47"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="41"/>
+    </row>
+    <row r="51" spans="1:3" ht="32" customHeight="1">
+      <c r="A51" s="47"/>
+      <c r="B51" s="44"/>
+      <c r="C51" s="41"/>
+    </row>
+    <row r="52" spans="1:3" ht="48" customHeight="1">
+      <c r="A52" s="47"/>
+      <c r="B52" s="44"/>
+      <c r="C52" s="41"/>
+    </row>
+    <row r="53" spans="1:3" ht="48" customHeight="1">
+      <c r="A53" s="47"/>
+      <c r="B53" s="44"/>
+      <c r="C53" s="41"/>
+    </row>
+    <row r="54" spans="1:3" ht="32" customHeight="1">
+      <c r="A54" s="47"/>
+      <c r="B54" s="44"/>
+      <c r="C54" s="41"/>
+    </row>
+    <row r="55" spans="1:3" ht="64" customHeight="1">
+      <c r="A55" s="47"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="41"/>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="47"/>
+      <c r="B56" s="44"/>
+      <c r="C56" s="41"/>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="47"/>
+      <c r="B57" s="44"/>
+      <c r="C57" s="41"/>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="47"/>
+      <c r="B58" s="44"/>
+      <c r="C58" s="41"/>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="47"/>
+      <c r="B59" s="44"/>
+      <c r="C59" s="41"/>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="47"/>
+      <c r="B60" s="44"/>
+      <c r="C60" s="41"/>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="47"/>
+      <c r="B61" s="44"/>
+      <c r="C61" s="41"/>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="47"/>
+      <c r="B62" s="44"/>
+      <c r="C62" s="41"/>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="47"/>
+      <c r="B63" s="44"/>
+      <c r="C63" s="41"/>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="47"/>
+      <c r="B64" s="44"/>
+      <c r="C64" s="41"/>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" s="47"/>
+      <c r="B65" s="44"/>
+      <c r="C65" s="41"/>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" s="47"/>
+      <c r="B66" s="44"/>
+      <c r="C66" s="41"/>
+    </row>
+    <row r="67" spans="1:3">
+      <c r="A67" s="47"/>
+      <c r="B67" s="44"/>
+      <c r="C67" s="41"/>
+    </row>
+    <row r="68" spans="1:3">
+      <c r="A68" s="47"/>
+      <c r="B68" s="44"/>
+      <c r="C68" s="41"/>
+    </row>
+    <row r="69" spans="1:3">
+      <c r="A69" s="47"/>
+      <c r="B69" s="45"/>
+      <c r="C69" s="41"/>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" s="47"/>
+      <c r="B70" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C44" s="63"/>
-    </row>
-    <row r="45" spans="1:3" ht="64" customHeight="1">
-      <c r="A45" s="37"/>
-      <c r="B45" s="38"/>
-      <c r="C45" s="64"/>
-    </row>
-    <row r="46" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A46" s="36" t="s">
-        <v>190</v>
-      </c>
-      <c r="B46" s="38"/>
-      <c r="C46" s="62" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" ht="64" customHeight="1">
-      <c r="A47" s="39"/>
-      <c r="B47" s="38"/>
-      <c r="C47" s="63"/>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" s="39"/>
-      <c r="B48" s="38"/>
-      <c r="C48" s="63"/>
-    </row>
-    <row r="49" spans="1:3" ht="48" customHeight="1">
-      <c r="A49" s="39"/>
-      <c r="B49" s="38"/>
-      <c r="C49" s="63"/>
-    </row>
-    <row r="50" spans="1:3" ht="48" customHeight="1">
-      <c r="A50" s="39"/>
-      <c r="B50" s="38"/>
-      <c r="C50" s="63"/>
-    </row>
-    <row r="51" spans="1:3" ht="32" customHeight="1">
-      <c r="A51" s="39"/>
-      <c r="B51" s="38"/>
-      <c r="C51" s="63"/>
-    </row>
-    <row r="52" spans="1:3" ht="48" customHeight="1">
-      <c r="A52" s="39"/>
-      <c r="B52" s="38"/>
-      <c r="C52" s="63"/>
-    </row>
-    <row r="53" spans="1:3" ht="48" customHeight="1">
-      <c r="A53" s="39"/>
-      <c r="B53" s="38"/>
-      <c r="C53" s="63"/>
-    </row>
-    <row r="54" spans="1:3" ht="32" customHeight="1">
-      <c r="A54" s="39"/>
-      <c r="B54" s="38"/>
-      <c r="C54" s="63"/>
-    </row>
-    <row r="55" spans="1:3" ht="64" customHeight="1">
-      <c r="A55" s="39"/>
-      <c r="B55" s="38"/>
-      <c r="C55" s="63"/>
-    </row>
-    <row r="56" spans="1:3">
-      <c r="A56" s="39"/>
-      <c r="B56" s="38"/>
-      <c r="C56" s="63"/>
-    </row>
-    <row r="57" spans="1:3">
-      <c r="A57" s="39"/>
-      <c r="B57" s="38"/>
-      <c r="C57" s="63"/>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" s="39"/>
-      <c r="B58" s="38"/>
-      <c r="C58" s="63"/>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" s="39"/>
-      <c r="B59" s="38"/>
-      <c r="C59" s="63"/>
-    </row>
-    <row r="60" spans="1:3">
-      <c r="A60" s="39"/>
-      <c r="B60" s="38"/>
-      <c r="C60" s="63"/>
-    </row>
-    <row r="61" spans="1:3">
-      <c r="A61" s="39"/>
-      <c r="B61" s="38"/>
-      <c r="C61" s="63"/>
-    </row>
-    <row r="62" spans="1:3">
-      <c r="A62" s="39"/>
-      <c r="B62" s="38"/>
-      <c r="C62" s="63"/>
-    </row>
-    <row r="63" spans="1:3">
-      <c r="A63" s="39"/>
-      <c r="B63" s="38"/>
-      <c r="C63" s="63"/>
-    </row>
-    <row r="64" spans="1:3">
-      <c r="A64" s="39"/>
-      <c r="B64" s="38"/>
-      <c r="C64" s="63"/>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" s="39"/>
-      <c r="B65" s="38"/>
-      <c r="C65" s="63"/>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" s="39"/>
-      <c r="B66" s="38"/>
-      <c r="C66" s="63"/>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" s="39"/>
-      <c r="B67" s="38"/>
-      <c r="C67" s="63"/>
-    </row>
-    <row r="68" spans="1:3">
-      <c r="A68" s="39"/>
-      <c r="B68" s="38"/>
-      <c r="C68" s="63"/>
-    </row>
-    <row r="69" spans="1:3">
-      <c r="A69" s="39"/>
-      <c r="B69" s="38"/>
-      <c r="C69" s="63"/>
-    </row>
-    <row r="70" spans="1:3">
-      <c r="A70" s="39"/>
-      <c r="B70" s="38"/>
-      <c r="C70" s="63"/>
+      <c r="C70" s="41"/>
     </row>
     <row r="71" spans="1:3">
-      <c r="A71" s="39"/>
-      <c r="B71" s="35"/>
-      <c r="C71" s="63"/>
+      <c r="A71" s="47"/>
+      <c r="B71" s="44"/>
+      <c r="C71" s="41"/>
     </row>
     <row r="72" spans="1:3">
-      <c r="A72" s="39"/>
-      <c r="B72" s="34" t="s">
+      <c r="A72" s="47"/>
+      <c r="B72" s="44"/>
+      <c r="C72" s="41"/>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" s="48"/>
+      <c r="B73" s="44"/>
+      <c r="C73" s="42"/>
+    </row>
+    <row r="74" spans="1:3" ht="409.5" customHeight="1">
+      <c r="A74" s="46" t="s">
+        <v>191</v>
+      </c>
+      <c r="B74" s="44"/>
+      <c r="C74" s="40" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="80" customHeight="1">
+      <c r="A75" s="47"/>
+      <c r="B75" s="44"/>
+      <c r="C75" s="41"/>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" s="47"/>
+      <c r="B76" s="44"/>
+      <c r="C76" s="41"/>
+    </row>
+    <row r="77" spans="1:3" ht="48" customHeight="1">
+      <c r="A77" s="47"/>
+      <c r="B77" s="44"/>
+      <c r="C77" s="41"/>
+    </row>
+    <row r="78" spans="1:3" ht="48" customHeight="1">
+      <c r="A78" s="47"/>
+      <c r="B78" s="44"/>
+      <c r="C78" s="41"/>
+    </row>
+    <row r="79" spans="1:3" ht="48" customHeight="1">
+      <c r="A79" s="47"/>
+      <c r="B79" s="44"/>
+      <c r="C79" s="41"/>
+    </row>
+    <row r="80" spans="1:3" ht="32" customHeight="1">
+      <c r="A80" s="47"/>
+      <c r="B80" s="44"/>
+      <c r="C80" s="41"/>
+    </row>
+    <row r="81" spans="1:3" ht="64" customHeight="1">
+      <c r="A81" s="47"/>
+      <c r="B81" s="44"/>
+      <c r="C81" s="41"/>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" s="47"/>
+      <c r="B82" s="44"/>
+      <c r="C82" s="41"/>
+    </row>
+    <row r="83" spans="1:3" ht="32" customHeight="1">
+      <c r="A83" s="47"/>
+      <c r="B83" s="44"/>
+      <c r="C83" s="41"/>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="47"/>
+      <c r="B84" s="44"/>
+      <c r="C84" s="41"/>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="47"/>
+      <c r="B85" s="44"/>
+      <c r="C85" s="41"/>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" s="47"/>
+      <c r="B86" s="44"/>
+      <c r="C86" s="41"/>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" s="47"/>
+      <c r="B87" s="44"/>
+      <c r="C87" s="41"/>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" s="47"/>
+      <c r="B88" s="44"/>
+      <c r="C88" s="41"/>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" s="47"/>
+      <c r="B89" s="44"/>
+      <c r="C89" s="41"/>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" s="47"/>
+      <c r="B90" s="44"/>
+      <c r="C90" s="41"/>
+    </row>
+    <row r="91" spans="1:3">
+      <c r="A91" s="47"/>
+      <c r="B91" s="44"/>
+      <c r="C91" s="41"/>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" s="47"/>
+      <c r="B92" s="44"/>
+      <c r="C92" s="41"/>
+    </row>
+    <row r="93" spans="1:3">
+      <c r="A93" s="47"/>
+      <c r="B93" s="44"/>
+      <c r="C93" s="41"/>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="47"/>
+      <c r="B94" s="44"/>
+      <c r="C94" s="41"/>
+    </row>
+    <row r="95" spans="1:3">
+      <c r="A95" s="47"/>
+      <c r="B95" s="44"/>
+      <c r="C95" s="41"/>
+    </row>
+    <row r="96" spans="1:3">
+      <c r="A96" s="47"/>
+      <c r="B96" s="44"/>
+      <c r="C96" s="41"/>
+    </row>
+    <row r="97" spans="1:3">
+      <c r="A97" s="47"/>
+      <c r="B97" s="44"/>
+      <c r="C97" s="41"/>
+    </row>
+    <row r="98" spans="1:3">
+      <c r="A98" s="47"/>
+      <c r="B98" s="45"/>
+      <c r="C98" s="41"/>
+    </row>
+    <row r="99" spans="1:3">
+      <c r="A99" s="47"/>
+      <c r="B99" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C72" s="63"/>
-    </row>
-    <row r="73" spans="1:3">
-      <c r="A73" s="37"/>
-      <c r="B73" s="38"/>
-      <c r="C73" s="64"/>
-    </row>
-    <row r="74" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A74" s="36" t="s">
-        <v>191</v>
-      </c>
-      <c r="B74" s="38"/>
-      <c r="C74" s="62" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="80" customHeight="1">
-      <c r="A75" s="39"/>
-      <c r="B75" s="38"/>
-      <c r="C75" s="63"/>
-    </row>
-    <row r="76" spans="1:3">
-      <c r="A76" s="39"/>
-      <c r="B76" s="38"/>
-      <c r="C76" s="63"/>
-    </row>
-    <row r="77" spans="1:3" ht="48" customHeight="1">
-      <c r="A77" s="39"/>
-      <c r="B77" s="38"/>
-      <c r="C77" s="63"/>
-    </row>
-    <row r="78" spans="1:3" ht="48" customHeight="1">
-      <c r="A78" s="39"/>
-      <c r="B78" s="38"/>
-      <c r="C78" s="63"/>
-    </row>
-    <row r="79" spans="1:3" ht="48" customHeight="1">
-      <c r="A79" s="39"/>
-      <c r="B79" s="38"/>
-      <c r="C79" s="63"/>
-    </row>
-    <row r="80" spans="1:3" ht="32" customHeight="1">
-      <c r="A80" s="39"/>
-      <c r="B80" s="38"/>
-      <c r="C80" s="63"/>
-    </row>
-    <row r="81" spans="1:3" ht="64" customHeight="1">
-      <c r="A81" s="39"/>
-      <c r="B81" s="38"/>
-      <c r="C81" s="63"/>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82" s="39"/>
-      <c r="B82" s="38"/>
-      <c r="C82" s="63"/>
-    </row>
-    <row r="83" spans="1:3" ht="32" customHeight="1">
-      <c r="A83" s="39"/>
-      <c r="B83" s="38"/>
-      <c r="C83" s="63"/>
-    </row>
-    <row r="84" spans="1:3">
-      <c r="A84" s="39"/>
-      <c r="B84" s="38"/>
-      <c r="C84" s="63"/>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85" s="39"/>
-      <c r="B85" s="38"/>
-      <c r="C85" s="63"/>
-    </row>
-    <row r="86" spans="1:3">
-      <c r="A86" s="39"/>
-      <c r="B86" s="38"/>
-      <c r="C86" s="63"/>
-    </row>
-    <row r="87" spans="1:3">
-      <c r="A87" s="39"/>
-      <c r="B87" s="38"/>
-      <c r="C87" s="63"/>
-    </row>
-    <row r="88" spans="1:3">
-      <c r="A88" s="39"/>
-      <c r="B88" s="38"/>
-      <c r="C88" s="63"/>
-    </row>
-    <row r="89" spans="1:3">
-      <c r="A89" s="39"/>
-      <c r="B89" s="38"/>
-      <c r="C89" s="63"/>
-    </row>
-    <row r="90" spans="1:3">
-      <c r="A90" s="39"/>
-      <c r="B90" s="38"/>
-      <c r="C90" s="63"/>
-    </row>
-    <row r="91" spans="1:3">
-      <c r="A91" s="39"/>
-      <c r="B91" s="38"/>
-      <c r="C91" s="63"/>
-    </row>
-    <row r="92" spans="1:3">
-      <c r="A92" s="39"/>
-      <c r="B92" s="38"/>
-      <c r="C92" s="63"/>
-    </row>
-    <row r="93" spans="1:3">
-      <c r="A93" s="39"/>
-      <c r="B93" s="38"/>
-      <c r="C93" s="63"/>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" s="39"/>
-      <c r="B94" s="38"/>
-      <c r="C94" s="63"/>
-    </row>
-    <row r="95" spans="1:3">
-      <c r="A95" s="39"/>
-      <c r="B95" s="38"/>
-      <c r="C95" s="63"/>
-    </row>
-    <row r="96" spans="1:3">
-      <c r="A96" s="39"/>
-      <c r="B96" s="38"/>
-      <c r="C96" s="63"/>
-    </row>
-    <row r="97" spans="1:3">
-      <c r="A97" s="39"/>
-      <c r="B97" s="38"/>
-      <c r="C97" s="63"/>
-    </row>
-    <row r="98" spans="1:3">
-      <c r="A98" s="39"/>
-      <c r="B98" s="38"/>
-      <c r="C98" s="63"/>
-    </row>
-    <row r="99" spans="1:3">
-      <c r="A99" s="39"/>
-      <c r="B99" s="38"/>
-      <c r="C99" s="63"/>
+      <c r="C99" s="41"/>
     </row>
     <row r="100" spans="1:3">
-      <c r="A100" s="39"/>
-      <c r="B100" s="35"/>
-      <c r="C100" s="63"/>
+      <c r="A100" s="47"/>
+      <c r="B100" s="44"/>
+      <c r="C100" s="41"/>
     </row>
     <row r="101" spans="1:3">
-      <c r="A101" s="39"/>
-      <c r="B101" s="34" t="s">
+      <c r="A101" s="47"/>
+      <c r="B101" s="44"/>
+      <c r="C101" s="41"/>
+    </row>
+    <row r="102" spans="1:3">
+      <c r="A102" s="48"/>
+      <c r="B102" s="44"/>
+      <c r="C102" s="42"/>
+    </row>
+    <row r="103" spans="1:3" ht="409.5" customHeight="1">
+      <c r="A103" s="46" t="s">
+        <v>192</v>
+      </c>
+      <c r="B103" s="44"/>
+      <c r="C103" s="40" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" ht="80" customHeight="1">
+      <c r="A104" s="47"/>
+      <c r="B104" s="44"/>
+      <c r="C104" s="41"/>
+    </row>
+    <row r="105" spans="1:3">
+      <c r="A105" s="47"/>
+      <c r="B105" s="44"/>
+      <c r="C105" s="41"/>
+    </row>
+    <row r="106" spans="1:3" ht="64" customHeight="1">
+      <c r="A106" s="47"/>
+      <c r="B106" s="44"/>
+      <c r="C106" s="41"/>
+    </row>
+    <row r="107" spans="1:3" ht="64" customHeight="1">
+      <c r="A107" s="47"/>
+      <c r="B107" s="44"/>
+      <c r="C107" s="41"/>
+    </row>
+    <row r="108" spans="1:3" ht="48" customHeight="1">
+      <c r="A108" s="47"/>
+      <c r="B108" s="44"/>
+      <c r="C108" s="41"/>
+    </row>
+    <row r="109" spans="1:3">
+      <c r="A109" s="47"/>
+      <c r="B109" s="44"/>
+      <c r="C109" s="41"/>
+    </row>
+    <row r="110" spans="1:3" ht="32" customHeight="1">
+      <c r="A110" s="47"/>
+      <c r="B110" s="44"/>
+      <c r="C110" s="41"/>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" s="47"/>
+      <c r="B111" s="44"/>
+      <c r="C111" s="41"/>
+    </row>
+    <row r="112" spans="1:3">
+      <c r="A112" s="47"/>
+      <c r="B112" s="44"/>
+      <c r="C112" s="41"/>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" s="47"/>
+      <c r="B113" s="44"/>
+      <c r="C113" s="41"/>
+    </row>
+    <row r="114" spans="1:3">
+      <c r="A114" s="47"/>
+      <c r="B114" s="44"/>
+      <c r="C114" s="41"/>
+    </row>
+    <row r="115" spans="1:3">
+      <c r="A115" s="47"/>
+      <c r="B115" s="44"/>
+      <c r="C115" s="41"/>
+    </row>
+    <row r="116" spans="1:3">
+      <c r="A116" s="47"/>
+      <c r="B116" s="44"/>
+      <c r="C116" s="41"/>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" s="47"/>
+      <c r="B117" s="44"/>
+      <c r="C117" s="41"/>
+    </row>
+    <row r="118" spans="1:3">
+      <c r="A118" s="47"/>
+      <c r="B118" s="44"/>
+      <c r="C118" s="41"/>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" s="47"/>
+      <c r="B119" s="44"/>
+      <c r="C119" s="41"/>
+    </row>
+    <row r="120" spans="1:3">
+      <c r="A120" s="47"/>
+      <c r="B120" s="44"/>
+      <c r="C120" s="41"/>
+    </row>
+    <row r="121" spans="1:3">
+      <c r="A121" s="47"/>
+      <c r="B121" s="44"/>
+      <c r="C121" s="41"/>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" s="47"/>
+      <c r="B122" s="44"/>
+      <c r="C122" s="41"/>
+    </row>
+    <row r="123" spans="1:3">
+      <c r="A123" s="47"/>
+      <c r="B123" s="44"/>
+      <c r="C123" s="41"/>
+    </row>
+    <row r="124" spans="1:3">
+      <c r="A124" s="47"/>
+      <c r="B124" s="45"/>
+      <c r="C124" s="41"/>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" s="47"/>
+      <c r="B125" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="C101" s="63"/>
-    </row>
-    <row r="102" spans="1:3">
-      <c r="A102" s="37"/>
-      <c r="B102" s="38"/>
-      <c r="C102" s="64"/>
-    </row>
-    <row r="103" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A103" s="36" t="s">
-        <v>192</v>
-      </c>
-      <c r="B103" s="38"/>
-      <c r="C103" s="62" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" ht="80" customHeight="1">
-      <c r="A104" s="39"/>
-      <c r="B104" s="38"/>
-      <c r="C104" s="63"/>
-    </row>
-    <row r="105" spans="1:3">
-      <c r="A105" s="39"/>
-      <c r="B105" s="38"/>
-      <c r="C105" s="63"/>
-    </row>
-    <row r="106" spans="1:3" ht="64" customHeight="1">
-      <c r="A106" s="39"/>
-      <c r="B106" s="38"/>
-      <c r="C106" s="63"/>
-    </row>
-    <row r="107" spans="1:3" ht="64" customHeight="1">
-      <c r="A107" s="39"/>
-      <c r="B107" s="38"/>
-      <c r="C107" s="63"/>
-    </row>
-    <row r="108" spans="1:3" ht="48" customHeight="1">
-      <c r="A108" s="39"/>
-      <c r="B108" s="38"/>
-      <c r="C108" s="63"/>
-    </row>
-    <row r="109" spans="1:3">
-      <c r="A109" s="39"/>
-      <c r="B109" s="38"/>
-      <c r="C109" s="63"/>
-    </row>
-    <row r="110" spans="1:3" ht="32" customHeight="1">
-      <c r="A110" s="39"/>
-      <c r="B110" s="38"/>
-      <c r="C110" s="63"/>
-    </row>
-    <row r="111" spans="1:3">
-      <c r="A111" s="39"/>
-      <c r="B111" s="38"/>
-      <c r="C111" s="63"/>
-    </row>
-    <row r="112" spans="1:3">
-      <c r="A112" s="39"/>
-      <c r="B112" s="38"/>
-      <c r="C112" s="63"/>
-    </row>
-    <row r="113" spans="1:3">
-      <c r="A113" s="39"/>
-      <c r="B113" s="38"/>
-      <c r="C113" s="63"/>
-    </row>
-    <row r="114" spans="1:3">
-      <c r="A114" s="39"/>
-      <c r="B114" s="38"/>
-      <c r="C114" s="63"/>
-    </row>
-    <row r="115" spans="1:3">
-      <c r="A115" s="39"/>
-      <c r="B115" s="38"/>
-      <c r="C115" s="63"/>
-    </row>
-    <row r="116" spans="1:3">
-      <c r="A116" s="39"/>
-      <c r="B116" s="38"/>
-      <c r="C116" s="63"/>
-    </row>
-    <row r="117" spans="1:3">
-      <c r="A117" s="39"/>
-      <c r="B117" s="38"/>
-      <c r="C117" s="63"/>
-    </row>
-    <row r="118" spans="1:3">
-      <c r="A118" s="39"/>
-      <c r="B118" s="38"/>
-      <c r="C118" s="63"/>
-    </row>
-    <row r="119" spans="1:3">
-      <c r="A119" s="39"/>
-      <c r="B119" s="38"/>
-      <c r="C119" s="63"/>
-    </row>
-    <row r="120" spans="1:3">
-      <c r="A120" s="39"/>
-      <c r="B120" s="38"/>
-      <c r="C120" s="63"/>
-    </row>
-    <row r="121" spans="1:3">
-      <c r="A121" s="39"/>
-      <c r="B121" s="38"/>
-      <c r="C121" s="63"/>
-    </row>
-    <row r="122" spans="1:3">
-      <c r="A122" s="39"/>
-      <c r="B122" s="38"/>
-      <c r="C122" s="63"/>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" s="39"/>
-      <c r="B123" s="38"/>
-      <c r="C123" s="63"/>
-    </row>
-    <row r="124" spans="1:3">
-      <c r="A124" s="39"/>
-      <c r="B124" s="38"/>
-      <c r="C124" s="63"/>
-    </row>
-    <row r="125" spans="1:3">
-      <c r="A125" s="39"/>
-      <c r="B125" s="38"/>
-      <c r="C125" s="63"/>
+      <c r="C125" s="41"/>
     </row>
     <row r="126" spans="1:3">
-      <c r="A126" s="39"/>
-      <c r="B126" s="35"/>
-      <c r="C126" s="63"/>
+      <c r="A126" s="47"/>
+      <c r="B126" s="44"/>
+      <c r="C126" s="41"/>
     </row>
     <row r="127" spans="1:3">
-      <c r="A127" s="39"/>
-      <c r="B127" s="34" t="s">
-        <v>62</v>
-      </c>
-      <c r="C127" s="63"/>
+      <c r="A127" s="47"/>
+      <c r="B127" s="44"/>
+      <c r="C127" s="41"/>
     </row>
     <row r="128" spans="1:3">
-      <c r="A128" s="37"/>
-      <c r="B128" s="38"/>
-      <c r="C128" s="64"/>
+      <c r="A128" s="48"/>
+      <c r="B128" s="44"/>
+      <c r="C128" s="42"/>
     </row>
     <row r="129" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A129" s="36" t="s">
+      <c r="A129" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="B129" s="38"/>
-      <c r="C129" s="62" t="s">
+      <c r="B129" s="44"/>
+      <c r="C129" s="40" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="130" spans="1:3" ht="80" customHeight="1">
-      <c r="A130" s="39"/>
-      <c r="B130" s="38"/>
-      <c r="C130" s="63"/>
+      <c r="A130" s="47"/>
+      <c r="B130" s="44"/>
+      <c r="C130" s="41"/>
     </row>
     <row r="131" spans="1:3">
-      <c r="A131" s="39"/>
-      <c r="B131" s="38"/>
-      <c r="C131" s="63"/>
+      <c r="A131" s="47"/>
+      <c r="B131" s="44"/>
+      <c r="C131" s="41"/>
     </row>
     <row r="132" spans="1:3">
-      <c r="A132" s="39"/>
-      <c r="B132" s="38"/>
-      <c r="C132" s="63"/>
+      <c r="A132" s="47"/>
+      <c r="B132" s="44"/>
+      <c r="C132" s="41"/>
     </row>
     <row r="133" spans="1:3">
-      <c r="A133" s="39"/>
-      <c r="B133" s="38"/>
-      <c r="C133" s="63"/>
+      <c r="A133" s="47"/>
+      <c r="B133" s="44"/>
+      <c r="C133" s="41"/>
     </row>
     <row r="134" spans="1:3" ht="48" customHeight="1">
-      <c r="A134" s="39"/>
-      <c r="B134" s="38"/>
-      <c r="C134" s="63"/>
+      <c r="A134" s="47"/>
+      <c r="B134" s="44"/>
+      <c r="C134" s="41"/>
     </row>
     <row r="135" spans="1:3" ht="80" customHeight="1">
-      <c r="A135" s="39"/>
-      <c r="B135" s="38"/>
-      <c r="C135" s="63"/>
+      <c r="A135" s="47"/>
+      <c r="B135" s="44"/>
+      <c r="C135" s="41"/>
     </row>
     <row r="136" spans="1:3" ht="64" customHeight="1">
-      <c r="A136" s="39"/>
-      <c r="B136" s="38"/>
-      <c r="C136" s="63"/>
+      <c r="A136" s="47"/>
+      <c r="B136" s="44"/>
+      <c r="C136" s="41"/>
     </row>
     <row r="137" spans="1:3" ht="32" customHeight="1">
-      <c r="A137" s="39"/>
-      <c r="B137" s="38"/>
-      <c r="C137" s="63"/>
+      <c r="A137" s="47"/>
+      <c r="B137" s="45"/>
+      <c r="C137" s="41"/>
     </row>
     <row r="138" spans="1:3">
-      <c r="A138" s="39"/>
-      <c r="B138" s="38"/>
-      <c r="C138" s="63"/>
+      <c r="A138" s="47"/>
+      <c r="B138" s="61">
+        <v>11012044</v>
+      </c>
+      <c r="C138" s="41"/>
     </row>
     <row r="139" spans="1:3" ht="80" customHeight="1">
-      <c r="A139" s="39"/>
-      <c r="B139" s="35"/>
-      <c r="C139" s="63"/>
+      <c r="A139" s="47"/>
+      <c r="B139" s="62"/>
+      <c r="C139" s="41"/>
     </row>
     <row r="140" spans="1:3">
-      <c r="A140" s="39"/>
-      <c r="B140" s="55">
-        <v>11012044</v>
-      </c>
-      <c r="C140" s="63"/>
+      <c r="A140" s="47"/>
+      <c r="B140" s="62"/>
+      <c r="C140" s="41"/>
     </row>
     <row r="141" spans="1:3">
-      <c r="A141" s="37"/>
-      <c r="B141" s="56"/>
-      <c r="C141" s="64"/>
+      <c r="A141" s="48"/>
+      <c r="B141" s="62"/>
+      <c r="C141" s="42"/>
     </row>
     <row r="142" spans="1:3" ht="404" customHeight="1">
-      <c r="A142" s="36" t="s">
+      <c r="A142" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="B142" s="56"/>
-      <c r="C142" s="62" t="s">
+      <c r="B142" s="62"/>
+      <c r="C142" s="40" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="143" spans="1:3" ht="64" customHeight="1">
-      <c r="A143" s="39"/>
-      <c r="B143" s="56"/>
-      <c r="C143" s="63"/>
+      <c r="A143" s="47"/>
+      <c r="B143" s="62"/>
+      <c r="C143" s="41"/>
     </row>
     <row r="144" spans="1:3">
-      <c r="A144" s="39"/>
-      <c r="B144" s="56"/>
-      <c r="C144" s="63"/>
+      <c r="A144" s="47"/>
+      <c r="B144" s="62"/>
+      <c r="C144" s="41"/>
     </row>
     <row r="145" spans="1:3" ht="64" customHeight="1">
-      <c r="A145" s="39"/>
-      <c r="B145" s="56"/>
-      <c r="C145" s="63"/>
+      <c r="A145" s="47"/>
+      <c r="B145" s="62"/>
+      <c r="C145" s="41"/>
     </row>
     <row r="146" spans="1:3">
-      <c r="A146" s="39"/>
-      <c r="B146" s="56"/>
-      <c r="C146" s="63"/>
+      <c r="A146" s="47"/>
+      <c r="B146" s="62"/>
+      <c r="C146" s="41"/>
     </row>
     <row r="147" spans="1:3" ht="32" customHeight="1">
-      <c r="A147" s="39"/>
-      <c r="B147" s="56"/>
-      <c r="C147" s="63"/>
+      <c r="A147" s="47"/>
+      <c r="B147" s="62"/>
+      <c r="C147" s="41"/>
     </row>
     <row r="148" spans="1:3">
-      <c r="A148" s="39"/>
-      <c r="B148" s="56"/>
-      <c r="C148" s="63"/>
+      <c r="A148" s="47"/>
+      <c r="B148" s="62"/>
+      <c r="C148" s="41"/>
     </row>
     <row r="149" spans="1:3">
-      <c r="A149" s="39"/>
-      <c r="B149" s="56"/>
-      <c r="C149" s="63"/>
+      <c r="A149" s="47"/>
+      <c r="B149" s="62"/>
+      <c r="C149" s="41"/>
     </row>
     <row r="150" spans="1:3">
-      <c r="A150" s="39"/>
-      <c r="B150" s="56"/>
-      <c r="C150" s="63"/>
+      <c r="A150" s="47"/>
+      <c r="B150" s="62"/>
+      <c r="C150" s="41"/>
     </row>
     <row r="151" spans="1:3">
-      <c r="A151" s="39"/>
-      <c r="B151" s="56"/>
-      <c r="C151" s="63"/>
+      <c r="A151" s="47"/>
+      <c r="B151" s="62"/>
+      <c r="C151" s="41"/>
     </row>
     <row r="152" spans="1:3">
-      <c r="A152" s="39"/>
-      <c r="B152" s="56"/>
-      <c r="C152" s="63"/>
+      <c r="A152" s="47"/>
+      <c r="B152" s="62"/>
+      <c r="C152" s="41"/>
     </row>
     <row r="153" spans="1:3">
-      <c r="A153" s="39"/>
-      <c r="B153" s="56"/>
-      <c r="C153" s="63"/>
+      <c r="A153" s="47"/>
+      <c r="B153" s="63"/>
+      <c r="C153" s="41"/>
     </row>
     <row r="154" spans="1:3">
-      <c r="A154" s="39"/>
-      <c r="B154" s="56"/>
-      <c r="C154" s="63"/>
+      <c r="A154" s="47"/>
+      <c r="B154" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C154" s="41"/>
     </row>
     <row r="155" spans="1:3">
-      <c r="A155" s="39"/>
-      <c r="B155" s="57"/>
-      <c r="C155" s="63"/>
+      <c r="A155" s="47"/>
+      <c r="B155" s="44"/>
+      <c r="C155" s="41"/>
     </row>
     <row r="156" spans="1:3">
-      <c r="A156" s="39"/>
-      <c r="B156" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C156" s="63"/>
+      <c r="A156" s="47"/>
+      <c r="B156" s="45"/>
+      <c r="C156" s="41"/>
     </row>
     <row r="157" spans="1:3">
-      <c r="A157" s="37"/>
-      <c r="B157" s="38"/>
-      <c r="C157" s="64"/>
+      <c r="A157" s="48"/>
+      <c r="B157" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C157" s="42"/>
     </row>
     <row r="158" spans="1:3" ht="68" customHeight="1">
-      <c r="A158" s="36" t="s">
+      <c r="A158" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B158" s="35"/>
-      <c r="C158" s="62" t="s">
+      <c r="B158" s="45"/>
+      <c r="C158" s="40" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="159" spans="1:3" ht="32" customHeight="1">
-      <c r="A159" s="39"/>
-      <c r="B159" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C159" s="63"/>
+      <c r="A159" s="47"/>
+      <c r="B159" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C159" s="41"/>
     </row>
     <row r="160" spans="1:3">
-      <c r="A160" s="37"/>
-      <c r="B160" s="35"/>
-      <c r="C160" s="64"/>
+      <c r="A160" s="48"/>
+      <c r="B160" s="44"/>
+      <c r="C160" s="42"/>
     </row>
     <row r="161" spans="1:3" ht="32" customHeight="1">
-      <c r="A161" s="45" t="s">
+      <c r="A161" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="B161" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C161" s="65" t="s">
+      <c r="B161" s="44"/>
+      <c r="C161" s="38" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="162" spans="1:3">
-      <c r="A162" s="46"/>
-      <c r="B162" s="38"/>
-      <c r="C162" s="66"/>
+      <c r="A162" s="70"/>
+      <c r="B162" s="44"/>
+      <c r="C162" s="39"/>
     </row>
     <row r="163" spans="1:3" ht="221" customHeight="1">
-      <c r="A163" s="36" t="s">
+      <c r="A163" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="B163" s="38"/>
-      <c r="C163" s="62" t="s">
+      <c r="B163" s="44"/>
+      <c r="C163" s="40" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="164" spans="1:3" ht="48" customHeight="1">
-      <c r="A164" s="39"/>
-      <c r="B164" s="38"/>
-      <c r="C164" s="63"/>
+      <c r="A164" s="47"/>
+      <c r="B164" s="44"/>
+      <c r="C164" s="41"/>
     </row>
     <row r="165" spans="1:3">
-      <c r="A165" s="39"/>
-      <c r="B165" s="38"/>
-      <c r="C165" s="63"/>
+      <c r="A165" s="47"/>
+      <c r="B165" s="44"/>
+      <c r="C165" s="41"/>
     </row>
     <row r="166" spans="1:3">
-      <c r="A166" s="39"/>
-      <c r="B166" s="38"/>
-      <c r="C166" s="63"/>
+      <c r="A166" s="47"/>
+      <c r="B166" s="44"/>
+      <c r="C166" s="41"/>
     </row>
     <row r="167" spans="1:3" ht="32" customHeight="1">
-      <c r="A167" s="39"/>
-      <c r="B167" s="38"/>
-      <c r="C167" s="63"/>
+      <c r="A167" s="47"/>
+      <c r="B167" s="44"/>
+      <c r="C167" s="41"/>
     </row>
     <row r="168" spans="1:3" ht="32" customHeight="1">
-      <c r="A168" s="39"/>
-      <c r="B168" s="38"/>
-      <c r="C168" s="63"/>
+      <c r="A168" s="47"/>
+      <c r="B168" s="45"/>
+      <c r="C168" s="41"/>
     </row>
     <row r="169" spans="1:3">
-      <c r="A169" s="39"/>
-      <c r="B169" s="38"/>
-      <c r="C169" s="63"/>
+      <c r="A169" s="47"/>
+      <c r="B169" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C169" s="41"/>
     </row>
     <row r="170" spans="1:3">
-      <c r="A170" s="39"/>
-      <c r="B170" s="35"/>
-      <c r="C170" s="63"/>
+      <c r="A170" s="47"/>
+      <c r="B170" s="44"/>
+      <c r="C170" s="41"/>
     </row>
     <row r="171" spans="1:3">
-      <c r="A171" s="39"/>
-      <c r="B171" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C171" s="63"/>
+      <c r="A171" s="47"/>
+      <c r="B171" s="44"/>
+      <c r="C171" s="41"/>
     </row>
     <row r="172" spans="1:3">
-      <c r="A172" s="37"/>
-      <c r="B172" s="38"/>
-      <c r="C172" s="64"/>
+      <c r="A172" s="48"/>
+      <c r="B172" s="44"/>
+      <c r="C172" s="42"/>
     </row>
     <row r="173" spans="1:3" ht="238" customHeight="1">
-      <c r="A173" s="42" t="s">
+      <c r="A173" s="66" t="s">
         <v>26</v>
       </c>
-      <c r="B173" s="38"/>
-      <c r="C173" s="62" t="s">
+      <c r="B173" s="44"/>
+      <c r="C173" s="40" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="174" spans="1:3" ht="32" customHeight="1">
-      <c r="A174" s="43"/>
-      <c r="B174" s="38"/>
-      <c r="C174" s="63"/>
+      <c r="A174" s="67"/>
+      <c r="B174" s="44"/>
+      <c r="C174" s="41"/>
     </row>
     <row r="175" spans="1:3">
-      <c r="A175" s="43"/>
-      <c r="B175" s="38"/>
-      <c r="C175" s="63"/>
+      <c r="A175" s="67"/>
+      <c r="B175" s="45"/>
+      <c r="C175" s="41"/>
     </row>
     <row r="176" spans="1:3" ht="32" customHeight="1">
-      <c r="A176" s="43"/>
-      <c r="B176" s="38"/>
-      <c r="C176" s="63"/>
+      <c r="A176" s="67"/>
+      <c r="B176" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C176" s="41"/>
     </row>
     <row r="177" spans="1:3">
-      <c r="A177" s="43"/>
-      <c r="B177" s="35"/>
-      <c r="C177" s="63"/>
+      <c r="A177" s="67"/>
+      <c r="B177" s="44"/>
+      <c r="C177" s="41"/>
     </row>
     <row r="178" spans="1:3" ht="64" customHeight="1">
-      <c r="A178" s="43"/>
-      <c r="B178" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C178" s="63"/>
+      <c r="A178" s="67"/>
+      <c r="B178" s="44"/>
+      <c r="C178" s="41"/>
     </row>
     <row r="179" spans="1:3">
-      <c r="A179" s="44"/>
-      <c r="B179" s="38"/>
-      <c r="C179" s="64"/>
+      <c r="A179" s="68"/>
+      <c r="B179" s="44"/>
+      <c r="C179" s="42"/>
     </row>
     <row r="180" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A180" s="36" t="s">
+      <c r="A180" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="B180" s="38"/>
-      <c r="C180" s="62" t="s">
+      <c r="B180" s="44"/>
+      <c r="C180" s="40" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="181" spans="1:3" ht="48" customHeight="1">
-      <c r="A181" s="39"/>
-      <c r="B181" s="38"/>
-      <c r="C181" s="63"/>
+      <c r="A181" s="47"/>
+      <c r="B181" s="44"/>
+      <c r="C181" s="41"/>
     </row>
     <row r="182" spans="1:3">
-      <c r="A182" s="39"/>
-      <c r="B182" s="38"/>
-      <c r="C182" s="63"/>
+      <c r="A182" s="47"/>
+      <c r="B182" s="44"/>
+      <c r="C182" s="41"/>
     </row>
     <row r="183" spans="1:3" ht="64" customHeight="1">
-      <c r="A183" s="39"/>
-      <c r="B183" s="38"/>
-      <c r="C183" s="63"/>
+      <c r="A183" s="47"/>
+      <c r="B183" s="44"/>
+      <c r="C183" s="41"/>
     </row>
     <row r="184" spans="1:3">
-      <c r="A184" s="39"/>
-      <c r="B184" s="38"/>
-      <c r="C184" s="63"/>
+      <c r="A184" s="47"/>
+      <c r="B184" s="44"/>
+      <c r="C184" s="41"/>
     </row>
     <row r="185" spans="1:3">
-      <c r="A185" s="39"/>
-      <c r="B185" s="38"/>
-      <c r="C185" s="63"/>
+      <c r="A185" s="47"/>
+      <c r="B185" s="44"/>
+      <c r="C185" s="41"/>
     </row>
     <row r="186" spans="1:3">
-      <c r="A186" s="39"/>
-      <c r="B186" s="38"/>
-      <c r="C186" s="63"/>
+      <c r="A186" s="47"/>
+      <c r="B186" s="44"/>
+      <c r="C186" s="41"/>
     </row>
     <row r="187" spans="1:3">
-      <c r="A187" s="39"/>
-      <c r="B187" s="38"/>
-      <c r="C187" s="63"/>
+      <c r="A187" s="47"/>
+      <c r="B187" s="44"/>
+      <c r="C187" s="41"/>
     </row>
     <row r="188" spans="1:3">
-      <c r="A188" s="39"/>
-      <c r="B188" s="38"/>
-      <c r="C188" s="63"/>
+      <c r="A188" s="47"/>
+      <c r="B188" s="44"/>
+      <c r="C188" s="41"/>
     </row>
     <row r="189" spans="1:3">
-      <c r="A189" s="39"/>
-      <c r="B189" s="38"/>
-      <c r="C189" s="63"/>
+      <c r="A189" s="47"/>
+      <c r="B189" s="44"/>
+      <c r="C189" s="41"/>
     </row>
     <row r="190" spans="1:3">
-      <c r="A190" s="39"/>
-      <c r="B190" s="38"/>
-      <c r="C190" s="63"/>
+      <c r="A190" s="47"/>
+      <c r="B190" s="44"/>
+      <c r="C190" s="41"/>
     </row>
     <row r="191" spans="1:3">
-      <c r="A191" s="39"/>
-      <c r="B191" s="38"/>
-      <c r="C191" s="63"/>
+      <c r="A191" s="47"/>
+      <c r="B191" s="44"/>
+      <c r="C191" s="41"/>
     </row>
     <row r="192" spans="1:3">
-      <c r="A192" s="39"/>
-      <c r="B192" s="38"/>
-      <c r="C192" s="63"/>
+      <c r="A192" s="47"/>
+      <c r="B192" s="44"/>
+      <c r="C192" s="41"/>
     </row>
     <row r="193" spans="1:3">
-      <c r="A193" s="39"/>
-      <c r="B193" s="38"/>
-      <c r="C193" s="63"/>
+      <c r="A193" s="47"/>
+      <c r="B193" s="44"/>
+      <c r="C193" s="41"/>
     </row>
     <row r="194" spans="1:3">
-      <c r="A194" s="39"/>
-      <c r="B194" s="38"/>
-      <c r="C194" s="63"/>
+      <c r="A194" s="47"/>
+      <c r="B194" s="44"/>
+      <c r="C194" s="41"/>
     </row>
     <row r="195" spans="1:3">
-      <c r="A195" s="39"/>
-      <c r="B195" s="38"/>
-      <c r="C195" s="63"/>
+      <c r="A195" s="47"/>
+      <c r="B195" s="44"/>
+      <c r="C195" s="41"/>
     </row>
     <row r="196" spans="1:3">
-      <c r="A196" s="39"/>
-      <c r="B196" s="38"/>
-      <c r="C196" s="63"/>
+      <c r="A196" s="47"/>
+      <c r="B196" s="44"/>
+      <c r="C196" s="41"/>
     </row>
     <row r="197" spans="1:3">
-      <c r="A197" s="39"/>
-      <c r="B197" s="38"/>
-      <c r="C197" s="63"/>
+      <c r="A197" s="47"/>
+      <c r="B197" s="45"/>
+      <c r="C197" s="41"/>
     </row>
     <row r="198" spans="1:3">
-      <c r="A198" s="39"/>
-      <c r="B198" s="38"/>
-      <c r="C198" s="63"/>
+      <c r="A198" s="47"/>
+      <c r="B198" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C198" s="41"/>
     </row>
     <row r="199" spans="1:3">
-      <c r="A199" s="39"/>
-      <c r="B199" s="35"/>
-      <c r="C199" s="63"/>
+      <c r="A199" s="47"/>
+      <c r="B199" s="45"/>
+      <c r="C199" s="41"/>
     </row>
     <row r="200" spans="1:3">
-      <c r="A200" s="39"/>
-      <c r="B200" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C200" s="63"/>
+      <c r="A200" s="47"/>
+      <c r="B200" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C200" s="41"/>
     </row>
     <row r="201" spans="1:3">
-      <c r="A201" s="37"/>
-      <c r="B201" s="35"/>
-      <c r="C201" s="64"/>
+      <c r="A201" s="48"/>
+      <c r="B201" s="44"/>
+      <c r="C201" s="42"/>
     </row>
     <row r="202" spans="1:3" ht="48" customHeight="1">
-      <c r="A202" s="36" t="s">
+      <c r="A202" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="B202" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C202" s="65" t="s">
+      <c r="B202" s="44"/>
+      <c r="C202" s="38" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="203" spans="1:3">
-      <c r="A203" s="37"/>
-      <c r="B203" s="38"/>
-      <c r="C203" s="66"/>
+      <c r="A203" s="48"/>
+      <c r="B203" s="44"/>
+      <c r="C203" s="39"/>
     </row>
     <row r="204" spans="1:3" ht="255" customHeight="1">
-      <c r="A204" s="36" t="s">
+      <c r="A204" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="B204" s="38"/>
-      <c r="C204" s="62" t="s">
+      <c r="B204" s="44"/>
+      <c r="C204" s="40" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="205" spans="1:3" ht="96" customHeight="1">
-      <c r="A205" s="39"/>
-      <c r="B205" s="38"/>
-      <c r="C205" s="63"/>
+      <c r="A205" s="47"/>
+      <c r="B205" s="44"/>
+      <c r="C205" s="41"/>
     </row>
     <row r="206" spans="1:3">
-      <c r="A206" s="39"/>
-      <c r="B206" s="38"/>
-      <c r="C206" s="63"/>
+      <c r="A206" s="47"/>
+      <c r="B206" s="44"/>
+      <c r="C206" s="41"/>
     </row>
     <row r="207" spans="1:3" ht="32" customHeight="1">
-      <c r="A207" s="39"/>
-      <c r="B207" s="38"/>
-      <c r="C207" s="63"/>
+      <c r="A207" s="47"/>
+      <c r="B207" s="45"/>
+      <c r="C207" s="41"/>
     </row>
     <row r="208" spans="1:3">
-      <c r="A208" s="39"/>
-      <c r="B208" s="38"/>
-      <c r="C208" s="63"/>
+      <c r="A208" s="47"/>
+      <c r="B208" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C208" s="41"/>
     </row>
     <row r="209" spans="1:3">
-      <c r="A209" s="39"/>
-      <c r="B209" s="35"/>
-      <c r="C209" s="63"/>
+      <c r="A209" s="47"/>
+      <c r="B209" s="44"/>
+      <c r="C209" s="41"/>
     </row>
     <row r="210" spans="1:3">
-      <c r="A210" s="39"/>
-      <c r="B210" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C210" s="63"/>
+      <c r="A210" s="47"/>
+      <c r="B210" s="44"/>
+      <c r="C210" s="41"/>
     </row>
     <row r="211" spans="1:3">
-      <c r="A211" s="37"/>
-      <c r="B211" s="38"/>
-      <c r="C211" s="64"/>
+      <c r="A211" s="48"/>
+      <c r="B211" s="44"/>
+      <c r="C211" s="42"/>
     </row>
     <row r="212" spans="1:3" ht="255" customHeight="1">
-      <c r="A212" s="36" t="s">
+      <c r="A212" s="46" t="s">
         <v>196</v>
       </c>
-      <c r="B212" s="38"/>
-      <c r="C212" s="62" t="s">
+      <c r="B212" s="44"/>
+      <c r="C212" s="40" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="213" spans="1:3">
-      <c r="A213" s="39"/>
-      <c r="B213" s="38"/>
-      <c r="C213" s="63"/>
+      <c r="A213" s="47"/>
+      <c r="B213" s="44"/>
+      <c r="C213" s="41"/>
     </row>
     <row r="214" spans="1:3">
-      <c r="A214" s="39"/>
-      <c r="B214" s="38"/>
-      <c r="C214" s="63"/>
+      <c r="A214" s="47"/>
+      <c r="B214" s="44"/>
+      <c r="C214" s="41"/>
     </row>
     <row r="215" spans="1:3">
-      <c r="A215" s="39"/>
-      <c r="B215" s="38"/>
-      <c r="C215" s="63"/>
+      <c r="A215" s="47"/>
+      <c r="B215" s="44"/>
+      <c r="C215" s="41"/>
     </row>
     <row r="216" spans="1:3">
-      <c r="A216" s="39"/>
-      <c r="B216" s="38"/>
-      <c r="C216" s="63"/>
+      <c r="A216" s="47"/>
+      <c r="B216" s="44"/>
+      <c r="C216" s="41"/>
     </row>
     <row r="217" spans="1:3">
-      <c r="A217" s="39"/>
-      <c r="B217" s="38"/>
-      <c r="C217" s="63"/>
+      <c r="A217" s="47"/>
+      <c r="B217" s="44"/>
+      <c r="C217" s="41"/>
     </row>
     <row r="218" spans="1:3">
-      <c r="A218" s="39"/>
-      <c r="B218" s="38"/>
-      <c r="C218" s="63"/>
+      <c r="A218" s="47"/>
+      <c r="B218" s="44"/>
+      <c r="C218" s="41"/>
     </row>
     <row r="219" spans="1:3">
-      <c r="A219" s="39"/>
-      <c r="B219" s="38"/>
-      <c r="C219" s="63"/>
+      <c r="A219" s="47"/>
+      <c r="B219" s="45"/>
+      <c r="C219" s="41"/>
     </row>
     <row r="220" spans="1:3">
-      <c r="A220" s="39"/>
-      <c r="B220" s="38"/>
-      <c r="C220" s="63"/>
+      <c r="A220" s="47"/>
+      <c r="B220" s="43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C220" s="41"/>
     </row>
     <row r="221" spans="1:3">
-      <c r="A221" s="39"/>
-      <c r="B221" s="35"/>
-      <c r="C221" s="63"/>
+      <c r="A221" s="47"/>
+      <c r="B221" s="44"/>
+      <c r="C221" s="41"/>
     </row>
     <row r="222" spans="1:3">
-      <c r="A222" s="39"/>
-      <c r="B222" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="C222" s="63"/>
+      <c r="A222" s="47"/>
+      <c r="B222" s="44"/>
+      <c r="C222" s="41"/>
     </row>
     <row r="223" spans="1:3">
-      <c r="A223" s="37"/>
-      <c r="B223" s="38"/>
-      <c r="C223" s="64"/>
+      <c r="A223" s="48"/>
+      <c r="B223" s="45"/>
+      <c r="C223" s="42"/>
     </row>
     <row r="224" spans="1:3" ht="102" customHeight="1">
-      <c r="A224" s="36" t="s">
+      <c r="A224" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="B224" s="38"/>
-      <c r="C224" s="62" t="s">
+      <c r="B224" s="43" t="s">
+        <v>88</v>
+      </c>
+      <c r="C224" s="40" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="225" spans="1:3" ht="48" customHeight="1">
-      <c r="A225" s="39"/>
-      <c r="B225" s="35"/>
-      <c r="C225" s="63"/>
+      <c r="A225" s="47"/>
+      <c r="B225" s="44"/>
+      <c r="C225" s="41"/>
     </row>
     <row r="226" spans="1:3">
-      <c r="A226" s="39"/>
-      <c r="B226" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="C226" s="63"/>
+      <c r="A226" s="47"/>
+      <c r="B226" s="44"/>
+      <c r="C226" s="41"/>
     </row>
     <row r="227" spans="1:3">
-      <c r="A227" s="37"/>
-      <c r="B227" s="38"/>
-      <c r="C227" s="64"/>
+      <c r="A227" s="48"/>
+      <c r="B227" s="44"/>
+      <c r="C227" s="42"/>
     </row>
     <row r="228" spans="1:3" ht="409.5" customHeight="1">
-      <c r="A228" s="36" t="s">
+      <c r="A228" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="B228" s="38"/>
-      <c r="C228" s="62" t="s">
+      <c r="B228" s="44"/>
+      <c r="C228" s="40" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="229" spans="1:3" ht="32" customHeight="1">
-      <c r="A229" s="39"/>
-      <c r="B229" s="38"/>
-      <c r="C229" s="63"/>
+      <c r="A229" s="47"/>
+      <c r="B229" s="44"/>
+      <c r="C229" s="41"/>
     </row>
     <row r="230" spans="1:3">
-      <c r="A230" s="39"/>
-      <c r="B230" s="38"/>
-      <c r="C230" s="63"/>
+      <c r="A230" s="47"/>
+      <c r="B230" s="44"/>
+      <c r="C230" s="41"/>
     </row>
     <row r="231" spans="1:3" ht="48" customHeight="1">
-      <c r="A231" s="39"/>
-      <c r="B231" s="38"/>
-      <c r="C231" s="63"/>
+      <c r="A231" s="47"/>
+      <c r="B231" s="44"/>
+      <c r="C231" s="41"/>
     </row>
     <row r="232" spans="1:3" ht="48" customHeight="1">
-      <c r="A232" s="39"/>
-      <c r="B232" s="38"/>
-      <c r="C232" s="63"/>
+      <c r="A232" s="47"/>
+      <c r="B232" s="44"/>
+      <c r="C232" s="41"/>
     </row>
     <row r="233" spans="1:3" ht="64" customHeight="1">
-      <c r="A233" s="39"/>
-      <c r="B233" s="38"/>
-      <c r="C233" s="63"/>
+      <c r="A233" s="47"/>
+      <c r="B233" s="44"/>
+      <c r="C233" s="41"/>
     </row>
     <row r="234" spans="1:3" ht="48" customHeight="1">
-      <c r="A234" s="39"/>
-      <c r="B234" s="38"/>
-      <c r="C234" s="63"/>
+      <c r="A234" s="47"/>
+      <c r="B234" s="44"/>
+      <c r="C234" s="41"/>
     </row>
     <row r="235" spans="1:3" ht="48" customHeight="1">
-      <c r="A235" s="39"/>
-      <c r="B235" s="38"/>
-      <c r="C235" s="63"/>
+      <c r="A235" s="47"/>
+      <c r="B235" s="44"/>
+      <c r="C235" s="41"/>
     </row>
     <row r="236" spans="1:3">
-      <c r="A236" s="39"/>
-      <c r="B236" s="38"/>
-      <c r="C236" s="63"/>
+      <c r="A236" s="47"/>
+      <c r="B236" s="44"/>
+      <c r="C236" s="41"/>
     </row>
     <row r="237" spans="1:3">
-      <c r="A237" s="39"/>
-      <c r="B237" s="38"/>
-      <c r="C237" s="63"/>
+      <c r="A237" s="47"/>
+      <c r="B237" s="44"/>
+      <c r="C237" s="41"/>
     </row>
     <row r="238" spans="1:3">
-      <c r="A238" s="39"/>
-      <c r="B238" s="38"/>
-      <c r="C238" s="63"/>
+      <c r="A238" s="47"/>
+      <c r="B238" s="44"/>
+      <c r="C238" s="41"/>
     </row>
     <row r="239" spans="1:3" ht="32" customHeight="1">
-      <c r="A239" s="39"/>
-      <c r="B239" s="38"/>
-      <c r="C239" s="63"/>
+      <c r="A239" s="47"/>
+      <c r="B239" s="44"/>
+      <c r="C239" s="41"/>
     </row>
     <row r="240" spans="1:3" ht="32" customHeight="1">
-      <c r="A240" s="39"/>
-      <c r="B240" s="38"/>
-      <c r="C240" s="63"/>
+      <c r="A240" s="47"/>
+      <c r="B240" s="45"/>
+      <c r="C240" s="41"/>
     </row>
     <row r="241" spans="1:3" ht="32" customHeight="1">
-      <c r="A241" s="39"/>
-      <c r="B241" s="38"/>
-      <c r="C241" s="63"/>
+      <c r="A241" s="47"/>
+      <c r="B241" s="53">
+        <v>15472</v>
+      </c>
+      <c r="C241" s="41"/>
     </row>
     <row r="242" spans="1:3" ht="32" customHeight="1">
-      <c r="A242" s="39"/>
-      <c r="B242" s="35"/>
-      <c r="C242" s="63"/>
+      <c r="A242" s="47"/>
+      <c r="B242" s="54"/>
+      <c r="C242" s="41"/>
     </row>
     <row r="243" spans="1:3" ht="32" customHeight="1">
-      <c r="A243" s="39"/>
-      <c r="B243" s="47">
-        <v>15472</v>
-      </c>
-      <c r="C243" s="63"/>
+      <c r="A243" s="47"/>
+      <c r="B243" s="54"/>
+      <c r="C243" s="41"/>
     </row>
     <row r="244" spans="1:3">
-      <c r="A244" s="37"/>
-      <c r="B244" s="48"/>
-      <c r="C244" s="64"/>
+      <c r="A244" s="48"/>
+      <c r="B244" s="54"/>
+      <c r="C244" s="42"/>
     </row>
     <row r="245" spans="1:3" ht="289" customHeight="1">
-      <c r="A245" s="50" t="s">
+      <c r="A245" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="B245" s="48"/>
-      <c r="C245" s="62" t="s">
+      <c r="B245" s="54"/>
+      <c r="C245" s="40" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="80" customHeight="1">
-      <c r="A246" s="51"/>
-      <c r="B246" s="48"/>
-      <c r="C246" s="63"/>
+      <c r="A246" s="57"/>
+      <c r="B246" s="54"/>
+      <c r="C246" s="41"/>
     </row>
     <row r="247" spans="1:3">
-      <c r="A247" s="51"/>
-      <c r="B247" s="48"/>
-      <c r="C247" s="63"/>
+      <c r="A247" s="57"/>
+      <c r="B247" s="54"/>
+      <c r="C247" s="41"/>
     </row>
     <row r="248" spans="1:3">
-      <c r="A248" s="51"/>
-      <c r="B248" s="48"/>
-      <c r="C248" s="63"/>
+      <c r="A248" s="57"/>
+      <c r="B248" s="54"/>
+      <c r="C248" s="41"/>
     </row>
     <row r="249" spans="1:3">
-      <c r="A249" s="51"/>
-      <c r="B249" s="48"/>
-      <c r="C249" s="63"/>
+      <c r="A249" s="57"/>
+      <c r="B249" s="54"/>
+      <c r="C249" s="41"/>
     </row>
     <row r="250" spans="1:3" ht="32" customHeight="1">
-      <c r="A250" s="51"/>
-      <c r="B250" s="48"/>
-      <c r="C250" s="63"/>
+      <c r="A250" s="57"/>
+      <c r="B250" s="55"/>
+      <c r="C250" s="41"/>
     </row>
     <row r="251" spans="1:3" ht="32" customHeight="1">
-      <c r="A251" s="51"/>
-      <c r="B251" s="48"/>
-      <c r="C251" s="63"/>
+      <c r="A251" s="57"/>
+      <c r="B251" s="59">
+        <v>75009240</v>
+      </c>
+      <c r="C251" s="41"/>
     </row>
     <row r="252" spans="1:3" ht="32" customHeight="1">
-      <c r="A252" s="51"/>
-      <c r="B252" s="49"/>
-      <c r="C252" s="63"/>
+      <c r="A252" s="57"/>
+      <c r="B252" s="60"/>
+      <c r="C252" s="41"/>
     </row>
     <row r="253" spans="1:3">
-      <c r="A253" s="51"/>
-      <c r="B253" s="53">
-        <v>75009240</v>
-      </c>
-      <c r="C253" s="63"/>
+      <c r="A253" s="57"/>
+      <c r="B253" s="43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C253" s="41"/>
     </row>
     <row r="254" spans="1:3">
-      <c r="A254" s="52"/>
-      <c r="B254" s="54"/>
-      <c r="C254" s="64"/>
+      <c r="A254" s="58"/>
+      <c r="B254" s="44"/>
+      <c r="C254" s="42"/>
     </row>
     <row r="255" spans="1:3">
-      <c r="A255" s="40" t="s">
+      <c r="A255" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="B255" s="34" t="s">
-        <v>198</v>
-      </c>
-      <c r="C255" s="65" t="s">
+      <c r="B255" s="44"/>
+      <c r="C255" s="38" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="256" spans="1:3">
-      <c r="A256" s="41"/>
-      <c r="B256" s="38"/>
-      <c r="C256" s="66"/>
+      <c r="A256" s="65"/>
+      <c r="B256" s="44"/>
+      <c r="C256" s="39"/>
     </row>
     <row r="257" spans="1:3" ht="388" customHeight="1">
-      <c r="A257" s="36" t="s">
+      <c r="A257" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="B257" s="38"/>
-      <c r="C257" s="62" t="s">
+      <c r="B257" s="44"/>
+      <c r="C257" s="40" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="258" spans="1:3">
-      <c r="A258" s="39"/>
-      <c r="B258" s="38"/>
-      <c r="C258" s="63"/>
+      <c r="A258" s="47"/>
+      <c r="B258" s="44"/>
+      <c r="C258" s="41"/>
     </row>
     <row r="259" spans="1:3">
-      <c r="A259" s="39"/>
-      <c r="B259" s="38"/>
-      <c r="C259" s="63"/>
+      <c r="A259" s="47"/>
+      <c r="B259" s="44"/>
+      <c r="C259" s="41"/>
     </row>
     <row r="260" spans="1:3" ht="48" customHeight="1">
-      <c r="A260" s="39"/>
-      <c r="B260" s="38"/>
-      <c r="C260" s="63"/>
+      <c r="A260" s="47"/>
+      <c r="B260" s="44"/>
+      <c r="C260" s="41"/>
     </row>
     <row r="261" spans="1:3" ht="32" customHeight="1">
-      <c r="A261" s="39"/>
-      <c r="B261" s="38"/>
-      <c r="C261" s="63"/>
+      <c r="A261" s="47"/>
+      <c r="B261" s="44"/>
+      <c r="C261" s="41"/>
     </row>
     <row r="262" spans="1:3" ht="32" customHeight="1">
-      <c r="A262" s="39"/>
-      <c r="B262" s="38"/>
-      <c r="C262" s="63"/>
+      <c r="A262" s="47"/>
+      <c r="B262" s="44"/>
+      <c r="C262" s="41"/>
     </row>
     <row r="263" spans="1:3" ht="32" customHeight="1">
-      <c r="A263" s="39"/>
-      <c r="B263" s="38"/>
-      <c r="C263" s="63"/>
+      <c r="A263" s="47"/>
+      <c r="B263" s="44"/>
+      <c r="C263" s="41"/>
     </row>
     <row r="264" spans="1:3">
-      <c r="A264" s="39"/>
-      <c r="B264" s="38"/>
-      <c r="C264" s="63"/>
+      <c r="A264" s="47"/>
+      <c r="B264" s="44"/>
+      <c r="C264" s="41"/>
     </row>
     <row r="265" spans="1:3">
-      <c r="A265" s="39"/>
-      <c r="B265" s="38"/>
-      <c r="C265" s="63"/>
+      <c r="A265" s="47"/>
+      <c r="B265" s="44"/>
+      <c r="C265" s="41"/>
     </row>
     <row r="266" spans="1:3">
-      <c r="A266" s="39"/>
-      <c r="B266" s="38"/>
-      <c r="C266" s="63"/>
+      <c r="A266" s="47"/>
+      <c r="B266" s="44"/>
+      <c r="C266" s="41"/>
     </row>
     <row r="267" spans="1:3">
-      <c r="A267" s="39"/>
-      <c r="B267" s="38"/>
-      <c r="C267" s="63"/>
+      <c r="A267" s="47"/>
+      <c r="B267" s="44"/>
+      <c r="C267" s="41"/>
     </row>
     <row r="268" spans="1:3">
-      <c r="A268" s="39"/>
-      <c r="B268" s="38"/>
-      <c r="C268" s="63"/>
+      <c r="A268" s="47"/>
+      <c r="B268" s="45"/>
+      <c r="C268" s="41"/>
     </row>
     <row r="269" spans="1:3">
-      <c r="A269" s="39"/>
-      <c r="B269" s="38"/>
-      <c r="C269" s="63"/>
+      <c r="A269" s="47"/>
+      <c r="B269" s="43" t="s">
+        <v>78</v>
+      </c>
+      <c r="C269" s="41"/>
     </row>
     <row r="270" spans="1:3">
-      <c r="A270" s="39"/>
-      <c r="B270" s="35"/>
-      <c r="C270" s="63"/>
+      <c r="A270" s="47"/>
+      <c r="B270" s="44"/>
+      <c r="C270" s="41"/>
     </row>
     <row r="271" spans="1:3">
-      <c r="A271" s="39"/>
-      <c r="B271" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="C271" s="63"/>
+      <c r="A271" s="47"/>
+      <c r="B271" s="44"/>
+      <c r="C271" s="41"/>
     </row>
     <row r="272" spans="1:3">
-      <c r="A272" s="37"/>
-      <c r="B272" s="38"/>
-      <c r="C272" s="64"/>
+      <c r="A272" s="48"/>
+      <c r="B272" s="44"/>
+      <c r="C272" s="42"/>
     </row>
     <row r="273" spans="1:3" ht="306" customHeight="1">
-      <c r="A273" s="34" t="s">
+      <c r="A273" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="B273" s="38"/>
-      <c r="C273" s="62" t="s">
+      <c r="B273" s="44"/>
+      <c r="C273" s="40" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="274" spans="1:3">
-      <c r="A274" s="38"/>
-      <c r="B274" s="38"/>
-      <c r="C274" s="63"/>
+      <c r="A274" s="44"/>
+      <c r="B274" s="44"/>
+      <c r="C274" s="41"/>
     </row>
     <row r="275" spans="1:3" ht="48" customHeight="1">
-      <c r="A275" s="38"/>
-      <c r="B275" s="38"/>
-      <c r="C275" s="63"/>
+      <c r="A275" s="44"/>
+      <c r="B275" s="44"/>
+      <c r="C275" s="41"/>
     </row>
     <row r="276" spans="1:3">
-      <c r="A276" s="38"/>
-      <c r="B276" s="38"/>
-      <c r="C276" s="63"/>
+      <c r="A276" s="44"/>
+      <c r="B276" s="44"/>
+      <c r="C276" s="41"/>
     </row>
     <row r="277" spans="1:3">
-      <c r="A277" s="38"/>
-      <c r="B277" s="38"/>
-      <c r="C277" s="63"/>
+      <c r="A277" s="44"/>
+      <c r="B277" s="44"/>
+      <c r="C277" s="41"/>
     </row>
     <row r="278" spans="1:3">
-      <c r="A278" s="38"/>
-      <c r="B278" s="38"/>
-      <c r="C278" s="63"/>
+      <c r="A278" s="44"/>
+      <c r="B278" s="44"/>
+      <c r="C278" s="41"/>
     </row>
     <row r="279" spans="1:3">
-      <c r="A279" s="38"/>
-      <c r="B279" s="38"/>
-      <c r="C279" s="63"/>
+      <c r="A279" s="44"/>
+      <c r="B279" s="44"/>
+      <c r="C279" s="41"/>
     </row>
     <row r="280" spans="1:3" ht="32" customHeight="1">
-      <c r="A280" s="38"/>
-      <c r="B280" s="38"/>
-      <c r="C280" s="63"/>
+      <c r="A280" s="44"/>
+      <c r="B280" s="44"/>
+      <c r="C280" s="41"/>
     </row>
     <row r="281" spans="1:3">
-      <c r="A281" s="38"/>
-      <c r="B281" s="38"/>
-      <c r="C281" s="63"/>
+      <c r="A281" s="44"/>
+      <c r="B281" s="44"/>
+      <c r="C281" s="41"/>
     </row>
     <row r="282" spans="1:3">
-      <c r="A282" s="38"/>
-      <c r="B282" s="38"/>
-      <c r="C282" s="63"/>
+      <c r="A282" s="44"/>
+      <c r="B282" s="44"/>
+      <c r="C282" s="41"/>
     </row>
     <row r="283" spans="1:3">
-      <c r="A283" s="38"/>
-      <c r="B283" s="38"/>
-      <c r="C283" s="63"/>
+      <c r="A283" s="44"/>
+      <c r="B283" s="45"/>
+      <c r="C283" s="41"/>
     </row>
     <row r="284" spans="1:3">
-      <c r="A284" s="38"/>
-      <c r="B284" s="38"/>
-      <c r="C284" s="63"/>
+      <c r="A284" s="44"/>
+      <c r="C284" s="41"/>
     </row>
     <row r="285" spans="1:3">
-      <c r="A285" s="38"/>
-      <c r="B285" s="35"/>
-      <c r="C285" s="63"/>
+      <c r="A285" s="44"/>
+      <c r="C285" s="41"/>
     </row>
     <row r="286" spans="1:3">
-      <c r="A286" s="38"/>
-      <c r="C286" s="63"/>
+      <c r="A286" s="44"/>
+      <c r="C286" s="41"/>
     </row>
     <row r="287" spans="1:3">
-      <c r="A287" s="38"/>
-      <c r="C287" s="64"/>
+      <c r="A287" s="44"/>
+      <c r="C287" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="77">
-    <mergeCell ref="C255:C256"/>
-    <mergeCell ref="C257:C272"/>
-    <mergeCell ref="C273:C287"/>
-    <mergeCell ref="C202:C203"/>
-    <mergeCell ref="C204:C211"/>
-    <mergeCell ref="C212:C223"/>
-    <mergeCell ref="C224:C227"/>
-    <mergeCell ref="C228:C244"/>
-    <mergeCell ref="C245:C254"/>
+  <mergeCells count="78">
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="A255:A256"/>
+    <mergeCell ref="B224:B240"/>
+    <mergeCell ref="A228:A244"/>
+    <mergeCell ref="B176:B197"/>
+    <mergeCell ref="A180:A201"/>
+    <mergeCell ref="B198:B199"/>
+    <mergeCell ref="A202:A203"/>
+    <mergeCell ref="A173:A179"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="A161:A162"/>
+    <mergeCell ref="B159:B168"/>
+    <mergeCell ref="A163:A172"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B241:B250"/>
+    <mergeCell ref="A245:A254"/>
+    <mergeCell ref="B251:B252"/>
+    <mergeCell ref="B169:B175"/>
+    <mergeCell ref="B125:B137"/>
+    <mergeCell ref="A129:A141"/>
+    <mergeCell ref="B138:B153"/>
+    <mergeCell ref="A142:A157"/>
+    <mergeCell ref="B99:B124"/>
+    <mergeCell ref="A103:A128"/>
+    <mergeCell ref="B9:B15"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B16:B30"/>
+    <mergeCell ref="B31:B41"/>
+    <mergeCell ref="A35:A45"/>
+    <mergeCell ref="B42:B69"/>
+    <mergeCell ref="A46:A73"/>
+    <mergeCell ref="B70:B98"/>
+    <mergeCell ref="A74:A102"/>
+    <mergeCell ref="A20:A34"/>
+    <mergeCell ref="B253:B268"/>
+    <mergeCell ref="A257:A272"/>
+    <mergeCell ref="B269:B283"/>
+    <mergeCell ref="A273:A287"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="B200:B207"/>
+    <mergeCell ref="A204:A211"/>
+    <mergeCell ref="B208:B219"/>
+    <mergeCell ref="A212:A223"/>
+    <mergeCell ref="B220:B223"/>
+    <mergeCell ref="A224:A227"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="A158:A160"/>
     <mergeCell ref="C180:C201"/>
     <mergeCell ref="C13:C19"/>
     <mergeCell ref="C35:C45"/>
@@ -7990,61 +8043,15 @@
     <mergeCell ref="C161:C162"/>
     <mergeCell ref="C163:C172"/>
     <mergeCell ref="C173:C179"/>
-    <mergeCell ref="B255:B270"/>
-    <mergeCell ref="A257:A272"/>
-    <mergeCell ref="B271:B285"/>
-    <mergeCell ref="A273:A287"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C8:C12"/>
-    <mergeCell ref="B202:B209"/>
-    <mergeCell ref="A204:A211"/>
-    <mergeCell ref="B210:B221"/>
-    <mergeCell ref="A212:A223"/>
-    <mergeCell ref="B222:B225"/>
-    <mergeCell ref="A224:A227"/>
-    <mergeCell ref="B156:B158"/>
-    <mergeCell ref="A158:A160"/>
-    <mergeCell ref="B33:B43"/>
-    <mergeCell ref="A35:A45"/>
-    <mergeCell ref="B44:B71"/>
-    <mergeCell ref="A46:A73"/>
-    <mergeCell ref="B72:B100"/>
-    <mergeCell ref="A74:A102"/>
-    <mergeCell ref="A20:A34"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B243:B252"/>
-    <mergeCell ref="A245:A254"/>
-    <mergeCell ref="B253:B254"/>
-    <mergeCell ref="B171:B177"/>
-    <mergeCell ref="B127:B139"/>
-    <mergeCell ref="A129:A141"/>
-    <mergeCell ref="B140:B155"/>
-    <mergeCell ref="A142:A157"/>
-    <mergeCell ref="B101:B126"/>
-    <mergeCell ref="A103:A128"/>
-    <mergeCell ref="B11:B17"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B18:B32"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="A255:A256"/>
-    <mergeCell ref="B226:B242"/>
-    <mergeCell ref="A228:A244"/>
-    <mergeCell ref="B178:B199"/>
-    <mergeCell ref="A180:A201"/>
-    <mergeCell ref="B200:B201"/>
-    <mergeCell ref="A202:A203"/>
-    <mergeCell ref="A173:A179"/>
-    <mergeCell ref="B159:B160"/>
-    <mergeCell ref="A161:A162"/>
-    <mergeCell ref="B161:B170"/>
-    <mergeCell ref="A163:A172"/>
+    <mergeCell ref="C255:C256"/>
+    <mergeCell ref="C257:C272"/>
+    <mergeCell ref="C273:C287"/>
+    <mergeCell ref="C202:C203"/>
+    <mergeCell ref="C204:C211"/>
+    <mergeCell ref="C212:C223"/>
+    <mergeCell ref="C224:C227"/>
+    <mergeCell ref="C228:C244"/>
+    <mergeCell ref="C245:C254"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -8316,7 +8323,7 @@
       <c r="B24" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="67" t="s">
+      <c r="C24" s="35" t="s">
         <v>52</v>
       </c>
     </row>
@@ -8599,7 +8606,7 @@
       <c r="A50" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="B50" s="68" t="s">
+      <c r="B50" s="36" t="s">
         <v>54</v>
       </c>
       <c r="C50" s="10" t="s">
@@ -8772,7 +8779,7 @@
       </c>
     </row>
     <row r="66" spans="1:3" ht="85">
-      <c r="A66" s="69" t="s">
+      <c r="A66" s="37" t="s">
         <v>155</v>
       </c>
       <c r="B66" s="11" t="s">

</xml_diff>